<commit_message>
subdivision de las pruebas para poder realizar los analisis
</commit_message>
<xml_diff>
--- a/PC-ROBOT/Pruebas_Funcionales/resultados/M4/M4_Pick_And_Place.xlsx
+++ b/PC-ROBOT/Pruebas_Funcionales/resultados/M4/M4_Pick_And_Place.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro_M4" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NASA-TLX" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Registro_M4" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="NASA-TLX" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -627,7 +627,9 @@
       <c r="F10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="4" t="n"/>
+      <c r="G10" s="4" t="n">
+        <v>184</v>
+      </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -666,7 +668,9 @@
       <c r="F11" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G11" s="4" t="n"/>
+      <c r="G11" s="4" t="n">
+        <v>425</v>
+      </c>
       <c r="H11" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -705,7 +709,9 @@
       <c r="F12" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="4" t="n"/>
+      <c r="G12" s="4" t="n">
+        <v>283</v>
+      </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -744,7 +750,9 @@
       <c r="F13" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="4" t="n"/>
+      <c r="G13" s="4" t="n">
+        <v>220</v>
+      </c>
       <c r="H13" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -783,7 +791,9 @@
       <c r="F14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n"/>
+      <c r="G14" s="4" t="n">
+        <v>407</v>
+      </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -820,7 +830,9 @@
       <c r="F15" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="4" t="n"/>
+      <c r="G15" s="4" t="n">
+        <v>36</v>
+      </c>
       <c r="H15" s="4" t="n">
         <v>0</v>
       </c>
@@ -855,7 +867,9 @@
       <c r="F16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="4" t="n"/>
+      <c r="G16" s="4" t="n">
+        <v>71</v>
+      </c>
       <c r="H16" s="4" t="n">
         <v>50</v>
       </c>
@@ -890,7 +904,9 @@
       <c r="F17" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="4" t="n"/>
+      <c r="G17" s="4" t="n">
+        <v>167</v>
+      </c>
       <c r="H17" s="4" t="n">
         <v>10</v>
       </c>
@@ -925,7 +941,9 @@
       <c r="F18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="4" t="n"/>
+      <c r="G18" s="4" t="n">
+        <v>39</v>
+      </c>
       <c r="H18" s="4" t="n">
         <v>10</v>
       </c>
@@ -960,7 +978,9 @@
       <c r="F19" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="4" t="n"/>
+      <c r="G19" s="4" t="n">
+        <v>50</v>
+      </c>
       <c r="H19" s="4" t="n">
         <v>0</v>
       </c>
@@ -995,7 +1015,9 @@
       <c r="F20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="4" t="n"/>
+      <c r="G20" s="4" t="n">
+        <v>55</v>
+      </c>
       <c r="H20" s="4" t="n">
         <v>11</v>
       </c>
@@ -1030,7 +1052,9 @@
       <c r="F21" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G21" s="4" t="n"/>
+      <c r="G21" s="4" t="n">
+        <v>40</v>
+      </c>
       <c r="H21" s="4" t="n">
         <v>18</v>
       </c>
@@ -1065,7 +1089,9 @@
       <c r="F22" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="4" t="n"/>
+      <c r="G22" s="4" t="n">
+        <v>37</v>
+      </c>
       <c r="H22" s="4" t="n">
         <v>27</v>
       </c>
@@ -1100,7 +1126,9 @@
       <c r="F23" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="4" t="n"/>
+      <c r="G23" s="4" t="n">
+        <v>41</v>
+      </c>
       <c r="H23" s="4" t="n">
         <v>18</v>
       </c>
@@ -1135,7 +1163,9 @@
       <c r="F24" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G24" s="4" t="n"/>
+      <c r="G24" s="4" t="n">
+        <v>36</v>
+      </c>
       <c r="H24" s="4" t="n">
         <v>11</v>
       </c>
@@ -1172,7 +1202,9 @@
       <c r="F25" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G25" s="4" t="n"/>
+      <c r="G25" s="4" t="n">
+        <v>63</v>
+      </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1211,7 +1243,9 @@
       <c r="F26" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G26" s="4" t="n"/>
+      <c r="G26" s="4" t="n">
+        <v>141</v>
+      </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1250,7 +1284,9 @@
       <c r="F27" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G27" s="4" t="n"/>
+      <c r="G27" s="4" t="n">
+        <v>200</v>
+      </c>
       <c r="H27" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1289,7 +1325,9 @@
       <c r="F28" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G28" s="4" t="n"/>
+      <c r="G28" s="4" t="n">
+        <v>228</v>
+      </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1328,7 +1366,9 @@
       <c r="F29" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="4" t="n"/>
+      <c r="G29" s="4" t="n">
+        <v>256</v>
+      </c>
       <c r="H29" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1371,7 +1411,9 @@
       <c r="F30" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G30" s="4" t="n"/>
+      <c r="G30" s="4" t="n">
+        <v>167</v>
+      </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1410,7 +1452,9 @@
       <c r="F31" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G31" s="4" t="n"/>
+      <c r="G31" s="4" t="n">
+        <v>261</v>
+      </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1449,7 +1493,9 @@
       <c r="F32" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G32" s="4" t="n"/>
+      <c r="G32" s="4" t="n">
+        <v>196</v>
+      </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1488,7 +1534,9 @@
       <c r="F33" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G33" s="4" t="n"/>
+      <c r="G33" s="4" t="n">
+        <v>188</v>
+      </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1527,7 +1575,9 @@
       <c r="F34" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="G34" s="4" t="n"/>
+      <c r="G34" s="4" t="n">
+        <v>295</v>
+      </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1564,7 +1614,9 @@
       <c r="F35" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G35" s="4" t="n"/>
+      <c r="G35" s="4" t="n">
+        <v>196</v>
+      </c>
       <c r="H35" s="4" t="n">
         <v>7</v>
       </c>
@@ -1599,7 +1651,9 @@
       <c r="F36" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G36" s="4" t="n"/>
+      <c r="G36" s="4" t="n">
+        <v>156</v>
+      </c>
       <c r="H36" s="4" t="n">
         <v>31</v>
       </c>
@@ -1634,7 +1688,9 @@
       <c r="F37" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="4" t="n"/>
+      <c r="G37" s="4" t="n">
+        <v>115</v>
+      </c>
       <c r="H37" s="4" t="n">
         <v>20</v>
       </c>
@@ -1669,7 +1725,9 @@
       <c r="F38" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G38" s="4" t="n"/>
+      <c r="G38" s="4" t="n">
+        <v>179</v>
+      </c>
       <c r="H38" s="4" t="n">
         <v>5</v>
       </c>
@@ -1706,7 +1764,9 @@
       <c r="F39" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G39" s="4" t="n"/>
+      <c r="G39" s="4" t="n">
+        <v>40</v>
+      </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
           <t>-</t>
@@ -1787,29 +1847,27 @@
           <t>N1</t>
         </is>
       </c>
-      <c r="C43" s="3">
-        <f>COUNTIFS(B10:B39,A43,C10:C39,B43)</f>
-        <v/>
-      </c>
-      <c r="D43" s="3">
-        <f>AVERAGEIFS(D10:D39,B10:B39,A43,C10:C39,B43)</f>
-        <v/>
-      </c>
-      <c r="E43" s="3">
-        <f>AVERAGEIFS(E10:E39,B10:B39,A43,C10:C39,B43)</f>
-        <v/>
-      </c>
-      <c r="F43" s="3">
-        <f>AVERAGEIFS(G10:G39,B10:B39,A43,C10:C39,B43)</f>
-        <v/>
-      </c>
-      <c r="G43" s="3">
-        <f>AVERAGEIFS(H10:H39,B10:B39,A43,C10:C39,B43)</f>
-        <v/>
-      </c>
-      <c r="H43" s="3">
-        <f>AVERAGEIFS(J10:J39,B10:B39,A43,C10:C39,B43)</f>
-        <v/>
+      <c r="C43" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>30.2</v>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="n">
+        <v>41.8</v>
+      </c>
+      <c r="G43" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1823,29 +1881,31 @@
           <t>N3</t>
         </is>
       </c>
-      <c r="C44" s="3">
-        <f>COUNTIFS(B10:B39,A44,C10:C39,B44)</f>
-        <v/>
-      </c>
-      <c r="D44" s="3">
-        <f>AVERAGEIFS(D10:D39,B10:B39,A44,C10:C39,B44)</f>
-        <v/>
-      </c>
-      <c r="E44" s="3">
-        <f>AVERAGEIFS(E10:E39,B10:B39,A44,C10:C39,B44)</f>
-        <v/>
-      </c>
-      <c r="F44" s="3">
-        <f>AVERAGEIFS(G10:G39,B10:B39,A44,C10:C39,B44)</f>
-        <v/>
-      </c>
-      <c r="G44" s="3">
-        <f>AVERAGEIFS(H10:H39,B10:B39,A44,C10:C39,B44)</f>
-        <v/>
-      </c>
-      <c r="H44" s="3">
-        <f>AVERAGEIFS(J10:J39,B10:B39,A44,C10:C39,B44)</f>
-        <v/>
+      <c r="C44" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>177.6</v>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -1859,29 +1919,27 @@
           <t>N1</t>
         </is>
       </c>
-      <c r="C45" s="3">
-        <f>COUNTIFS(B10:B39,A45,C10:C39,B45)</f>
-        <v/>
-      </c>
-      <c r="D45" s="3">
-        <f>AVERAGEIFS(D10:D39,B10:B39,A45,C10:C39,B45)</f>
-        <v/>
-      </c>
-      <c r="E45" s="3">
-        <f>AVERAGEIFS(E10:E39,B10:B39,A45,C10:C39,B45)</f>
-        <v/>
-      </c>
-      <c r="F45" s="3">
-        <f>AVERAGEIFS(G10:G39,B10:B39,A45,C10:C39,B45)</f>
-        <v/>
-      </c>
-      <c r="G45" s="3">
-        <f>AVERAGEIFS(H10:H39,B10:B39,A45,C10:C39,B45)</f>
-        <v/>
-      </c>
-      <c r="H45" s="3">
-        <f>AVERAGEIFS(J10:J39,B10:B39,A45,C10:C39,B45)</f>
-        <v/>
+      <c r="C45" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>44.8</v>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>72.59999999999999</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
       </c>
     </row>
     <row r="46">
@@ -1895,29 +1953,31 @@
           <t>N3</t>
         </is>
       </c>
-      <c r="C46" s="3">
-        <f>COUNTIFS(B10:B39,A46,C10:C39,B46)</f>
-        <v/>
-      </c>
-      <c r="D46" s="3">
-        <f>AVERAGEIFS(D10:D39,B10:B39,A46,C10:C39,B46)</f>
-        <v/>
-      </c>
-      <c r="E46" s="3">
-        <f>AVERAGEIFS(E10:E39,B10:B39,A46,C10:C39,B46)</f>
-        <v/>
-      </c>
-      <c r="F46" s="3">
-        <f>AVERAGEIFS(G10:G39,B10:B39,A46,C10:C39,B46)</f>
-        <v/>
-      </c>
-      <c r="G46" s="3">
-        <f>AVERAGEIFS(H10:H39,B10:B39,A46,C10:C39,B46)</f>
-        <v/>
-      </c>
-      <c r="H46" s="3">
-        <f>AVERAGEIFS(J10:J39,B10:B39,A46,C10:C39,B46)</f>
-        <v/>
+      <c r="C46" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>303.8</v>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -1931,29 +1991,27 @@
           <t>N1</t>
         </is>
       </c>
-      <c r="C47" s="3">
-        <f>COUNTIFS(B10:B39,A47,C10:C39,B47)</f>
-        <v/>
-      </c>
-      <c r="D47" s="3">
-        <f>AVERAGEIFS(D10:D39,B10:B39,A47,C10:C39,B47)</f>
-        <v/>
-      </c>
-      <c r="E47" s="3">
-        <f>AVERAGEIFS(E10:E39,B10:B39,A47,C10:C39,B47)</f>
-        <v/>
-      </c>
-      <c r="F47" s="3">
-        <f>AVERAGEIFS(G10:G39,B10:B39,A47,C10:C39,B47)</f>
-        <v/>
-      </c>
-      <c r="G47" s="3">
-        <f>AVERAGEIFS(H10:H39,B10:B39,A47,C10:C39,B47)</f>
-        <v/>
-      </c>
-      <c r="H47" s="3">
-        <f>AVERAGEIFS(J10:J39,B10:B39,A47,C10:C39,B47)</f>
-        <v/>
+      <c r="C47" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D47" s="3" t="n">
+        <v>45.8</v>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="n">
+        <v>137.2</v>
+      </c>
+      <c r="G47" s="3" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>80%</t>
+        </is>
       </c>
     </row>
     <row r="48">
@@ -1967,29 +2025,31 @@
           <t>N3</t>
         </is>
       </c>
-      <c r="C48" s="3">
-        <f>COUNTIFS(B10:B39,A48,C10:C39,B48)</f>
-        <v/>
-      </c>
-      <c r="D48" s="3">
-        <f>AVERAGEIFS(D10:D39,B10:B39,A48,C10:C39,B48)</f>
-        <v/>
-      </c>
-      <c r="E48" s="3">
-        <f>AVERAGEIFS(E10:E39,B10:B39,A48,C10:C39,B48)</f>
-        <v/>
-      </c>
-      <c r="F48" s="3">
-        <f>AVERAGEIFS(G10:G39,B10:B39,A48,C10:C39,B48)</f>
-        <v/>
-      </c>
-      <c r="G48" s="3">
-        <f>AVERAGEIFS(H10:H39,B10:B39,A48,C10:C39,B48)</f>
-        <v/>
-      </c>
-      <c r="H48" s="3">
-        <f>AVERAGEIFS(J10:J39,B10:B39,A48,C10:C39,B48)</f>
-        <v/>
+      <c r="C48" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>221.4</v>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
M4: rellenar Nº correcciones en las 30 filas a partir de correcciones_m4_completo_30_intentos.csv (eje dominante), emparejado por orden cronologico dentro de cada bloque objeto x condicion
</commit_message>
<xml_diff>
--- a/PC-ROBOT/Pruebas_Funcionales/resultados/M4/M4_Pick_And_Place.xlsx
+++ b/PC-ROBOT/Pruebas_Funcionales/resultados/M4/M4_Pick_And_Place.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Registro_M4" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="NASA-TLX" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registro_M4" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NASA-TLX" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -1780,10 +1780,10 @@
       </c>
       <c r="K39" s="4" t="n"/>
     </row>
-    <row r="40" ht="75" customHeight="1" s="6">
+    <row r="40" ht="95" customHeight="1" s="6">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Notas: (1) "-" indica que no aplica, no que el valor sea 0; se usa en Tiempo de compleción y Error de colocación cuando el intento no llegó a un evento de colocación medible (agarre fallido, o el objeto se cayó/perdió durante el transporte, p. ej. Nº 30). Las fórmulas AVERAGEIFS del resumen ignoran automáticamente estas celdas de texto. (2) La columna "Nº correcciones" queda sin rellenar en los 30 intentos: la intención era extraerla de los CSV funcionales con contador_correcciones.py, pero para no reiniciar la conexión WebRTC entre cada intento, el script se lanzó una sola vez por condición de red, así que id_intento se quedó fijo a 1 en todo el CSV de la sesión y no hay forma de aislar cada intento a posteriori. Corregido en safe8_WebRTC.py (25/08/2026): ahora, en sesiones M4, pulsar Enter en el terminal marca "siguiente intento" sin reiniciar la conexión, para que la próxima sesión física sí pueda rellenar esta columna.</t>
+          <t>Notas: (1) "-" indica que no aplica, no que el valor sea 0; se usa en Tiempo de compleción y Error de colocación cuando el intento no llegó a un evento de colocación medible (agarre fallido, o el objeto se cayó/perdió durante el transporte, p. ej. Nº 30). Las fórmulas AVERAGEIFS del resumen ignoran automáticamente estas celdas de texto. (2) "Nº correcciones" (25/08/2026): calculado con contador_correcciones.py (cambios de signo de la derivada en el eje dominante) sobre los CSV partidos por intento (N1_intentoN/N3_intentoN), generados aparte porque durante la sesión no se reinició la conexión entre cada intento y el CSV continuo no distinguía uno de otro (ver §10.9bis). El orden intento1..5 de esos CSV es cronológico y se ha emparejado en ese mismo orden con las filas de cada bloque objeto×condición; el recorte de cada intento es aproximado (puede incluir algo de margen antes o después del intento oficial), así que el número es una estimación de buena fe, no una medida perfectamente acotada al intento exacto.</t>
         </is>
       </c>
     </row>
@@ -1847,27 +1847,29 @@
           <t>N1</t>
         </is>
       </c>
-      <c r="C43" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D43" s="3" t="n">
-        <v>30.2</v>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>41.8</v>
-      </c>
-      <c r="G43" s="3" t="n">
-        <v>17</v>
-      </c>
-      <c r="H43" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
+      <c r="C43" s="3">
+        <f>COUNTIFS(B10:B39,A43,C10:C39,B43)</f>
+        <v/>
+      </c>
+      <c r="D43" s="3">
+        <f>AVERAGEIFS(D10:D39,B10:B39,A43,C10:C39,B43)</f>
+        <v/>
+      </c>
+      <c r="E43" s="3">
+        <f>AVERAGEIFS(E10:E39,B10:B39,A43,C10:C39,B43)</f>
+        <v/>
+      </c>
+      <c r="F43" s="3">
+        <f>AVERAGEIFS(G10:G39,B10:B39,A43,C10:C39,B43)</f>
+        <v/>
+      </c>
+      <c r="G43" s="3">
+        <f>AVERAGEIFS(H10:H39,B10:B39,A43,C10:C39,B43)</f>
+        <v/>
+      </c>
+      <c r="H43" s="3">
+        <f>AVERAGEIFS(J10:J39,B10:B39,A43,C10:C39,B43)</f>
+        <v/>
       </c>
     </row>
     <row r="44">
@@ -1881,31 +1883,29 @@
           <t>N3</t>
         </is>
       </c>
-      <c r="C44" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F44" s="3" t="n">
-        <v>177.6</v>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
+      <c r="C44" s="3">
+        <f>COUNTIFS(B10:B39,A44,C10:C39,B44)</f>
+        <v/>
+      </c>
+      <c r="D44" s="3">
+        <f>AVERAGEIFS(D10:D39,B10:B39,A44,C10:C39,B44)</f>
+        <v/>
+      </c>
+      <c r="E44" s="3">
+        <f>AVERAGEIFS(E10:E39,B10:B39,A44,C10:C39,B44)</f>
+        <v/>
+      </c>
+      <c r="F44" s="3">
+        <f>AVERAGEIFS(G10:G39,B10:B39,A44,C10:C39,B44)</f>
+        <v/>
+      </c>
+      <c r="G44" s="3">
+        <f>AVERAGEIFS(H10:H39,B10:B39,A44,C10:C39,B44)</f>
+        <v/>
+      </c>
+      <c r="H44" s="3">
+        <f>AVERAGEIFS(J10:J39,B10:B39,A44,C10:C39,B44)</f>
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1919,27 +1919,29 @@
           <t>N1</t>
         </is>
       </c>
-      <c r="C45" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D45" s="3" t="n">
-        <v>44.8</v>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="F45" s="3" t="n">
-        <v>72.59999999999999</v>
-      </c>
-      <c r="G45" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="H45" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
+      <c r="C45" s="3">
+        <f>COUNTIFS(B10:B39,A45,C10:C39,B45)</f>
+        <v/>
+      </c>
+      <c r="D45" s="3">
+        <f>AVERAGEIFS(D10:D39,B10:B39,A45,C10:C39,B45)</f>
+        <v/>
+      </c>
+      <c r="E45" s="3">
+        <f>AVERAGEIFS(E10:E39,B10:B39,A45,C10:C39,B45)</f>
+        <v/>
+      </c>
+      <c r="F45" s="3">
+        <f>AVERAGEIFS(G10:G39,B10:B39,A45,C10:C39,B45)</f>
+        <v/>
+      </c>
+      <c r="G45" s="3">
+        <f>AVERAGEIFS(H10:H39,B10:B39,A45,C10:C39,B45)</f>
+        <v/>
+      </c>
+      <c r="H45" s="3">
+        <f>AVERAGEIFS(J10:J39,B10:B39,A45,C10:C39,B45)</f>
+        <v/>
       </c>
     </row>
     <row r="46">
@@ -1953,31 +1955,29 @@
           <t>N3</t>
         </is>
       </c>
-      <c r="C46" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="n">
-        <v>303.8</v>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
+      <c r="C46" s="3">
+        <f>COUNTIFS(B10:B39,A46,C10:C39,B46)</f>
+        <v/>
+      </c>
+      <c r="D46" s="3">
+        <f>AVERAGEIFS(D10:D39,B10:B39,A46,C10:C39,B46)</f>
+        <v/>
+      </c>
+      <c r="E46" s="3">
+        <f>AVERAGEIFS(E10:E39,B10:B39,A46,C10:C39,B46)</f>
+        <v/>
+      </c>
+      <c r="F46" s="3">
+        <f>AVERAGEIFS(G10:G39,B10:B39,A46,C10:C39,B46)</f>
+        <v/>
+      </c>
+      <c r="G46" s="3">
+        <f>AVERAGEIFS(H10:H39,B10:B39,A46,C10:C39,B46)</f>
+        <v/>
+      </c>
+      <c r="H46" s="3">
+        <f>AVERAGEIFS(J10:J39,B10:B39,A46,C10:C39,B46)</f>
+        <v/>
       </c>
     </row>
     <row r="47">
@@ -1991,27 +1991,29 @@
           <t>N1</t>
         </is>
       </c>
-      <c r="C47" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D47" s="3" t="n">
-        <v>45.8</v>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="F47" s="3" t="n">
-        <v>137.2</v>
-      </c>
-      <c r="G47" s="3" t="n">
-        <v>15.8</v>
-      </c>
-      <c r="H47" s="3" t="inlineStr">
-        <is>
-          <t>80%</t>
-        </is>
+      <c r="C47" s="3">
+        <f>COUNTIFS(B10:B39,A47,C10:C39,B47)</f>
+        <v/>
+      </c>
+      <c r="D47" s="3">
+        <f>AVERAGEIFS(D10:D39,B10:B39,A47,C10:C39,B47)</f>
+        <v/>
+      </c>
+      <c r="E47" s="3">
+        <f>AVERAGEIFS(E10:E39,B10:B39,A47,C10:C39,B47)</f>
+        <v/>
+      </c>
+      <c r="F47" s="3">
+        <f>AVERAGEIFS(G10:G39,B10:B39,A47,C10:C39,B47)</f>
+        <v/>
+      </c>
+      <c r="G47" s="3">
+        <f>AVERAGEIFS(H10:H39,B10:B39,A47,C10:C39,B47)</f>
+        <v/>
+      </c>
+      <c r="H47" s="3">
+        <f>AVERAGEIFS(J10:J39,B10:B39,A47,C10:C39,B47)</f>
+        <v/>
       </c>
     </row>
     <row r="48">
@@ -2025,31 +2027,29 @@
           <t>N3</t>
         </is>
       </c>
-      <c r="C48" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-      <c r="F48" s="3" t="n">
-        <v>221.4</v>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
+      <c r="C48" s="3">
+        <f>COUNTIFS(B10:B39,A48,C10:C39,B48)</f>
+        <v/>
+      </c>
+      <c r="D48" s="3">
+        <f>AVERAGEIFS(D10:D39,B10:B39,A48,C10:C39,B48)</f>
+        <v/>
+      </c>
+      <c r="E48" s="3">
+        <f>AVERAGEIFS(E10:E39,B10:B39,A48,C10:C39,B48)</f>
+        <v/>
+      </c>
+      <c r="F48" s="3">
+        <f>AVERAGEIFS(G10:G39,B10:B39,A48,C10:C39,B48)</f>
+        <v/>
+      </c>
+      <c r="G48" s="3">
+        <f>AVERAGEIFS(H10:H39,B10:B39,A48,C10:C39,B48)</f>
+        <v/>
+      </c>
+      <c r="H48" s="3">
+        <f>AVERAGEIFS(J10:J39,B10:B39,A48,C10:C39,B48)</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>